<commit_message>
Kit Essencial: planilha 3 Ganhos e Gastos (lançamentos, painel, reserva, categorias, ano)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0146uBo6FVJ2cyEehyP8rK61
</commit_message>
<xml_diff>
--- a/projetos/gestao-ia-planilhas/produto/kit-essencial/02-relatorio-mensal-pronto.xlsx
+++ b/projetos/gestao-ia-planilhas/produto/kit-essencial/02-relatorio-mensal-pronto.xlsx
@@ -867,7 +867,7 @@
               </c:numCache>
             </c:numRef>
           </c:val>
-          <c:smooth val="1"/>
+          <c:smooth val="0"/>
         </c:ser>
         <c:ser>
           <c:idx val="1"/>
@@ -1006,7 +1006,7 @@
               </c:numCache>
             </c:numRef>
           </c:val>
-          <c:smooth val="1"/>
+          <c:smooth val="0"/>
         </c:ser>
         <c:hiLowLines>
           <c:spPr>
@@ -1016,11 +1016,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="81699257"/>
-        <c:axId val="57675937"/>
+        <c:axId val="43379599"/>
+        <c:axId val="69429372"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="81699257"/>
+        <c:axId val="43379599"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1052,7 +1052,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="57675937"/>
+        <c:crossAx val="69429372"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1060,7 +1060,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="57675937"/>
+        <c:axId val="69429372"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1092,7 +1092,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="81699257"/>
+        <c:crossAx val="43379599"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>

</xml_diff>